<commit_message>
Penyesuaian / fix form dan output image
</commit_message>
<xml_diff>
--- a/Laporan Buku Tamu.xlsx
+++ b/Laporan Buku Tamu.xlsx
@@ -41,16 +41,16 @@
     <t>2026-09-22</t>
   </si>
   <si>
-    <t>Reivan</t>
+    <t>irgi</t>
   </si>
   <si>
     <t>cianjur</t>
   </si>
   <si>
-    <t>08256778</t>
-  </si>
-  <si>
-    <t>Irgi</t>
+    <t>08123456</t>
+  </si>
+  <si>
+    <t>irfan</t>
   </si>
   <si>
     <t>Pribadi</t>

</xml_diff>